<commit_message>
Enhance Playwright tests: add stroke drawing verification and color functionality
</commit_message>
<xml_diff>
--- a/Docs/TestCases.xlsx
+++ b/Docs/TestCases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Main\source\repos\CollaborativeWhiteboard\Tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Main\source\repos\CollaborativeWhiteboard\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49182799-D70B-4B20-ACAC-28754668C2CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D20DCA7-7A02-47AD-A1A3-D829A295AE66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
add test case for verifying that user can change the rooms
</commit_message>
<xml_diff>
--- a/Docs/TestCases.xlsx
+++ b/Docs/TestCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Main\source\repos\CollaborativeWhiteboard\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D20DCA7-7A02-47AD-A1A3-D829A295AE66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4497992C-BF11-40E6-92FB-CA62A257B120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="50">
   <si>
     <t>ID</t>
   </si>
@@ -78,21 +78,9 @@
     <t>User B's canvas is also cleared</t>
   </si>
   <si>
-    <t>TC-09</t>
-  </si>
-  <si>
     <t>Room B remains unchanged</t>
   </si>
   <si>
-    <t>TC-10</t>
-  </si>
-  <si>
-    <t>User joins a room</t>
-  </si>
-  <si>
-    <t>User is connected to that room</t>
-  </si>
-  <si>
     <t>User changes from Room A to Room B</t>
   </si>
   <si>
@@ -168,12 +156,6 @@
     <t>User A clears Room A</t>
   </si>
   <si>
-    <t>User can join a room</t>
-  </si>
-  <si>
-    <t>App is running</t>
-  </si>
-  <si>
     <t>User can change rooms</t>
   </si>
   <si>
@@ -190,6 +172,9 @@
   </si>
   <si>
     <t>Both users see both strokes</t>
+  </si>
+  <si>
+    <t>TC-9</t>
   </si>
 </sst>
 </file>
@@ -542,19 +527,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -562,19 +547,19 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -582,19 +567,19 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -602,19 +587,19 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -622,19 +607,19 @@
         <v>6</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -642,10 +627,10 @@
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>9</v>
@@ -654,7 +639,7 @@
         <v>10</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -662,10 +647,10 @@
         <v>8</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>12</v>
@@ -674,7 +659,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -682,10 +667,10 @@
         <v>11</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>15</v>
@@ -694,7 +679,7 @@
         <v>16</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -702,61 +687,42 @@
         <v>14</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>

</xml_diff>